<commit_message>
G94-191: Align nutrition and kitchen screens with BA flow
- Add suppliers, purchase/stock unit conversion and dish duplication
- Allocate stock issues by lot and register meals from attendance
- Fix 422 when adding a dish to a weekly draft menu
- Rework weekly menu layout with separate allergy change rows
</commit_message>
<xml_diff>
--- a/public/templates/thuc-pham-mau.xlsx
+++ b/public/templates/thuc-pham-mau.xlsx
@@ -69,7 +69,7 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Bột</t>
+          <t>Tinh bột</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -128,7 +128,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kcal, Đạm, Béo, Bột: trên 100 g (hoặc 100 ml). Thải bỏ %: từ 0 đến 90.</t>
+          <t>Kcal, Đạm, Béo, Tinh bột: trên 100 g (hoặc 100 ml). Thải bỏ %: từ 0 đến 90.</t>
         </is>
       </c>
     </row>

</xml_diff>